<commit_message>
Daily screener update: 2026-07-07
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,312 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AMBQ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>APGE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BBGI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CLOV</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FTHM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IMUX</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>INHD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NMAD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>OTLK</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>QXL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RFL</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UMC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Initial</t>
         </is>
       </c>
     </row>
@@ -446,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,6 +769,91 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LUCY</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PEW</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SEER</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Initial</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-08
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -738,6 +738,244 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BFLY</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>GITS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>NIXX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>WNC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>XMTR</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>AMBQ</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BBGI</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IMUX</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>NMAD</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>QXL</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RFL</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>UMC</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -752,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -854,6 +1092,176 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CRNX</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WSO-B</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LUCY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PEW</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SEER</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
     </row>
@@ -868,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -888,6 +1296,40 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SNAL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-09
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1162,6 +1162,340 @@
         </is>
       </c>
       <c r="C33" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="G34" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="E35" t="n">
+        <v>46.71</v>
+      </c>
+      <c r="F35" t="n">
+        <v>72.18000000000001</v>
+      </c>
+      <c r="G35" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MGNX</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F36" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="G36" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MYSE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E37" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="F37" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="G37" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="F38" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="G38" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TWST</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>105.47</v>
+      </c>
+      <c r="E39" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>145.41</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>UMC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>28.96</v>
+      </c>
+      <c r="E40" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="F40" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="G40" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G41" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>BFLY</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CLOV</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GITS</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>OTLK</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>XMTR</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -1178,7 +1512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1525,6 +1859,161 @@
         </is>
       </c>
       <c r="C16" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EDBL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1712</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LUCY</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="G18" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G19" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CRNX</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>WSO-B</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -1541,7 +2030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1639,6 +2128,52 @@
         <v>78</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NVVE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="E4" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-9.15</v>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-10
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1496,6 +1496,364 @@
         </is>
       </c>
       <c r="C47" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BBGI</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>22.52</v>
+      </c>
+      <c r="F48" t="n">
+        <v>42.86</v>
+      </c>
+      <c r="G48" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>BFLY</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="E49" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="F49" t="n">
+        <v>14.64</v>
+      </c>
+      <c r="G49" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F50" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="G50" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>GITS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F51" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="G51" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>29.27</v>
+      </c>
+      <c r="E52" t="n">
+        <v>17.77</v>
+      </c>
+      <c r="F52" t="n">
+        <v>52.28</v>
+      </c>
+      <c r="G52" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PGEN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="E53" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F53" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="G53" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E54" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="F54" t="n">
+        <v>18.32</v>
+      </c>
+      <c r="G54" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>RNAC</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E55" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F55" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="G55" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>RRGB</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="E56" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F56" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="G56" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="E57" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="F57" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="G57" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>TWST</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -1512,7 +1870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2014,6 +2372,190 @@
         </is>
       </c>
       <c r="C23" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ALNY</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>380</v>
+      </c>
+      <c r="E24" t="n">
+        <v>311.1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>517.8</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="G25" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RKTO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="G26" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SMPL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="E27" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="F27" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G27" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EDBL</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LUCY</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -2030,7 +2572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2174,6 +2716,23 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SNAL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-11
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1854,6 +1854,345 @@
         </is>
       </c>
       <c r="C61" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ABSI</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="E62" t="n">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="F62" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="G62" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>AMPG</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="E63" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="F63" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="G63" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E64" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="F64" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G64" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>EVC</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="E65" t="n">
+        <v>11.05</v>
+      </c>
+      <c r="F65" t="n">
+        <v>19.12</v>
+      </c>
+      <c r="G65" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>GALT</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="E66" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F66" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="G66" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HSCS</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F67" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="G67" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="E68" t="n">
+        <v>81.15000000000001</v>
+      </c>
+      <c r="F68" t="n">
+        <v>131.04</v>
+      </c>
+      <c r="G68" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>INHD</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>MGNX</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>NIXX</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>RRGB</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>WNC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -1870,7 +2209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2556,6 +2895,161 @@
         </is>
       </c>
       <c r="C31" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ELAB</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="G33" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>WDFC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>298.9</v>
+      </c>
+      <c r="E34" t="n">
+        <v>261.49</v>
+      </c>
+      <c r="F34" t="n">
+        <v>373.72</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ALNY</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>RKTO</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SMPL</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-14
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2193,6 +2193,587 @@
         </is>
       </c>
       <c r="C76" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>13.59</v>
+      </c>
+      <c r="E77" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="F77" t="n">
+        <v>20.11</v>
+      </c>
+      <c r="G77" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>CLYM</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>14.41</v>
+      </c>
+      <c r="E78" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="F78" t="n">
+        <v>18.56</v>
+      </c>
+      <c r="G78" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>FLNT</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="E79" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F79" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="G79" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HPP</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E80" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="F80" t="n">
+        <v>21.66</v>
+      </c>
+      <c r="G80" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>IFRX</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F81" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="G81" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>OGN</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E82" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="F82" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="G82" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="E83" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="F83" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G83" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SLDB</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="E84" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="F84" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G84" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="E85" t="n">
+        <v>12</v>
+      </c>
+      <c r="F85" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="G85" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SOWG</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="E86" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="F86" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="G86" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>STTK</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E87" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="F87" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="G87" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>TWST</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>105.47</v>
+      </c>
+      <c r="E88" t="n">
+        <v>87.56999999999999</v>
+      </c>
+      <c r="F88" t="n">
+        <v>141.27</v>
+      </c>
+      <c r="G88" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="E89" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="F89" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="G89" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>AMPG</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BBGI</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>EVC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>FTHM</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>GALT</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>GITS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>HSCS</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>MYSE</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PGEN</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>RNAC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>UMC</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -2209,7 +2790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3050,6 +3631,202 @@
         </is>
       </c>
       <c r="C38" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AGEN</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="F39" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="G39" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BRAI</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="E40" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="F40" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="G40" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="E41" t="n">
+        <v>17.28</v>
+      </c>
+      <c r="F41" t="n">
+        <v>24.69</v>
+      </c>
+      <c r="G41" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SOBR</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>13.55</v>
+      </c>
+      <c r="E43" t="n">
+        <v>10.06</v>
+      </c>
+      <c r="F43" t="n">
+        <v>20.53</v>
+      </c>
+      <c r="G43" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ELAB</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>WDFC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -3066,7 +3843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3227,6 +4004,23 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NVVE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-15
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2774,6 +2774,374 @@
         </is>
       </c>
       <c r="C101" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>INHD</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>39.49</v>
+      </c>
+      <c r="E102" t="n">
+        <v>39.49</v>
+      </c>
+      <c r="F102" t="n">
+        <v>39.49</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>JXG</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>12</v>
+      </c>
+      <c r="E103" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="F103" t="n">
+        <v>14.62</v>
+      </c>
+      <c r="G103" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>66.55</v>
+      </c>
+      <c r="E104" t="n">
+        <v>52.51</v>
+      </c>
+      <c r="F104" t="n">
+        <v>94.63</v>
+      </c>
+      <c r="G104" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="E105" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F105" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="G105" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>RGNX</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="E106" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="F106" t="n">
+        <v>24.38</v>
+      </c>
+      <c r="G106" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>20.75</v>
+      </c>
+      <c r="E107" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="F107" t="n">
+        <v>36.21</v>
+      </c>
+      <c r="G107" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="E109" t="n">
+        <v>28.25</v>
+      </c>
+      <c r="F109" t="n">
+        <v>44.09</v>
+      </c>
+      <c r="G109" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>BFLY</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>IFRX</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>OGN</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SLDB</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>STTK</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -2790,7 +3158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3827,6 +4195,265 @@
         </is>
       </c>
       <c r="C46" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G47" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CLSK</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E48" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="F48" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="G48" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>LHAI</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G49" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="E50" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F50" t="n">
+        <v>14.31</v>
+      </c>
+      <c r="G50" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>NXTC</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="E51" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="F51" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="G51" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SHPH</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="E52" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F52" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="G52" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AGEN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>BRAI</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SOBR</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -3843,7 +4470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4021,6 +4648,35 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="E8" t="n">
+        <v>48.79</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-42.89</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-16
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3142,6 +3142,345 @@
         </is>
       </c>
       <c r="C117" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>574.2</v>
+      </c>
+      <c r="E118" t="n">
+        <v>498.15</v>
+      </c>
+      <c r="F118" t="n">
+        <v>726.3</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>BDSX</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>24.92</v>
+      </c>
+      <c r="E119" t="n">
+        <v>18.91</v>
+      </c>
+      <c r="F119" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="G119" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>BLZE</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="E120" t="n">
+        <v>14.52</v>
+      </c>
+      <c r="F120" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="G120" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="E121" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F121" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="G121" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>FTHM</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F122" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="G122" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>OGN</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E123" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="F123" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="G123" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>96.14</v>
+      </c>
+      <c r="E124" t="n">
+        <v>81.15000000000001</v>
+      </c>
+      <c r="F124" t="n">
+        <v>126.12</v>
+      </c>
+      <c r="G124" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>ABSI</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>CLYM</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>JXG</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>TNGX</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -3158,7 +3497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4454,6 +4793,369 @@
         </is>
       </c>
       <c r="C57" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>106.37</v>
+      </c>
+      <c r="E58" t="n">
+        <v>86.28</v>
+      </c>
+      <c r="F58" t="n">
+        <v>146.55</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ERNA</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E59" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="F59" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="G59" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G60" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>KUST</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F61" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="G61" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>54.73</v>
+      </c>
+      <c r="E62" t="n">
+        <v>53.44</v>
+      </c>
+      <c r="F62" t="n">
+        <v>57.31</v>
+      </c>
+      <c r="G62" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SLSN</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G63" t="n">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>SOBR</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="G64" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="E65" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F65" t="n">
+        <v>90.8</v>
+      </c>
+      <c r="G65" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>VIVS</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F66" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="G66" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>CLSK</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>LHAI</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>NXTC</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>SHPH</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -4470,7 +5172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4677,6 +5379,23 @@
         <v>1</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-17
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G132"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3481,6 +3481,471 @@
         </is>
       </c>
       <c r="C132" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>FATE</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E133" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F133" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="G133" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>GALT</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="E134" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F134" t="n">
+        <v>8.630000000000001</v>
+      </c>
+      <c r="G134" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>HNGE</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="E135" t="n">
+        <v>82.53</v>
+      </c>
+      <c r="F135" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="G135" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>HSCS</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E136" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="F136" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="G136" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E137" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="F137" t="n">
+        <v>18.28</v>
+      </c>
+      <c r="G137" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>RNAZ</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="E138" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F138" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="G138" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G139" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E140" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F140" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="G140" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="E141" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="F141" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="G141" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BDSX</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BLZE</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>FLNT</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>FTHM</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>HPP</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>OGN</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>RGNX</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -3497,7 +3962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5156,6 +5621,374 @@
         </is>
       </c>
       <c r="C72" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ATAI</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="E73" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="F73" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="G73" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ATPC</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="F74" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="G74" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>37.88</v>
+      </c>
+      <c r="E75" t="n">
+        <v>29.75</v>
+      </c>
+      <c r="F75" t="n">
+        <v>54.14</v>
+      </c>
+      <c r="G75" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>DSGR</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>34.83</v>
+      </c>
+      <c r="E76" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="F76" t="n">
+        <v>49.53</v>
+      </c>
+      <c r="G76" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>IQST</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F77" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="G77" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>LIMN</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1960</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="E79" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="F79" t="n">
+        <v>59.74</v>
+      </c>
+      <c r="G79" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>RUBI</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="E80" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="F80" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="G80" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ERNA</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>KUST</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SLSN</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SOBR</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>VIVS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-18
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3946,6 +3946,270 @@
         </is>
       </c>
       <c r="C153" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="E154" t="n">
+        <v>248.01</v>
+      </c>
+      <c r="F154" t="n">
+        <v>334.08</v>
+      </c>
+      <c r="G154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E155" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="F155" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G155" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>GITS</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="E156" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F156" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="G156" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>HPP</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E157" t="n">
+        <v>15.01</v>
+      </c>
+      <c r="F157" t="n">
+        <v>21.58</v>
+      </c>
+      <c r="G157" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>43.67</v>
+      </c>
+      <c r="E158" t="n">
+        <v>38</v>
+      </c>
+      <c r="F158" t="n">
+        <v>55.01</v>
+      </c>
+      <c r="G158" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>HNGE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>RNAZ</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>TWST</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -3962,7 +4226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5989,6 +6253,304 @@
         </is>
       </c>
       <c r="C88" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E89" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F89" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="G89" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G90" t="n">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>FFAI</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SDOT</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>25.14</v>
+      </c>
+      <c r="E92" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="F92" t="n">
+        <v>36.62</v>
+      </c>
+      <c r="G92" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E93" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="G93" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ATAI</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ATPC</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>DSGR</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>IQST</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>LIMN</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>RUBI</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-21
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G165"/>
+  <dimension ref="A1:G187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4210,6 +4210,536 @@
         </is>
       </c>
       <c r="C165" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>BWIN</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>28.55</v>
+      </c>
+      <c r="E166" t="n">
+        <v>25.55</v>
+      </c>
+      <c r="F166" t="n">
+        <v>34.55</v>
+      </c>
+      <c r="G166" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>CRNX</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>84</v>
+      </c>
+      <c r="E167" t="n">
+        <v>83.43000000000001</v>
+      </c>
+      <c r="F167" t="n">
+        <v>85.14</v>
+      </c>
+      <c r="G167" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="E168" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F168" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="G168" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="E169" t="n">
+        <v>8</v>
+      </c>
+      <c r="F169" t="n">
+        <v>13.32</v>
+      </c>
+      <c r="G169" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>FRMM</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>7</v>
+      </c>
+      <c r="E170" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="F170" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="G170" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>HNGE</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="E171" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="F171" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="G171" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>IMUX</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="E172" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="F172" t="n">
+        <v>19.26</v>
+      </c>
+      <c r="G172" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>MSLE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>10</v>
+      </c>
+      <c r="E173" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="F173" t="n">
+        <v>14.62</v>
+      </c>
+      <c r="G173" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>PTRN</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="E174" t="n">
+        <v>26.82</v>
+      </c>
+      <c r="F174" t="n">
+        <v>35.76</v>
+      </c>
+      <c r="G174" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="E175" t="n">
+        <v>18.33</v>
+      </c>
+      <c r="F175" t="n">
+        <v>25.71</v>
+      </c>
+      <c r="G175" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>20.75</v>
+      </c>
+      <c r="E176" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="F176" t="n">
+        <v>36.21</v>
+      </c>
+      <c r="G176" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>SDOT</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>55.88</v>
+      </c>
+      <c r="E177" t="n">
+        <v>11</v>
+      </c>
+      <c r="F177" t="n">
+        <v>145.64</v>
+      </c>
+      <c r="G177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="E178" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="F178" t="n">
+        <v>22.17</v>
+      </c>
+      <c r="G178" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>GALT</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>HPP</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>HSCS</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>SOWG</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -4226,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6551,6 +7081,178 @@
         </is>
       </c>
       <c r="C102" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="E103" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="F103" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="G103" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>AMC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="E104" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F104" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="G104" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>FGMC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E105" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="F105" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="G105" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>FFAI</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SDOT</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-22
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G187"/>
+  <dimension ref="A1:G206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4740,6 +4740,437 @@
         </is>
       </c>
       <c r="C187" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>ALIT</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>23.68</v>
+      </c>
+      <c r="E188" t="n">
+        <v>18.07</v>
+      </c>
+      <c r="F188" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="G188" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>14.59</v>
+      </c>
+      <c r="E189" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F189" t="n">
+        <v>32.77</v>
+      </c>
+      <c r="G189" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="E190" t="n">
+        <v>248.61</v>
+      </c>
+      <c r="F190" t="n">
+        <v>332.88</v>
+      </c>
+      <c r="G190" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="E191" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F191" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="G191" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="E192" t="n">
+        <v>18.02</v>
+      </c>
+      <c r="F192" t="n">
+        <v>24.03</v>
+      </c>
+      <c r="G192" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>157</v>
+      </c>
+      <c r="E193" t="n">
+        <v>134.37</v>
+      </c>
+      <c r="F193" t="n">
+        <v>202.26</v>
+      </c>
+      <c r="G193" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>RPD</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="E194" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="F194" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="G194" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>VRNS</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>49.54</v>
+      </c>
+      <c r="E195" t="n">
+        <v>43.74</v>
+      </c>
+      <c r="F195" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="G195" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E196" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F196" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="G196" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>APGE</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>FRMM</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>GITS</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>IMUX</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>PTRN</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>SDOT</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -4756,7 +5187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7253,6 +7684,318 @@
         </is>
       </c>
       <c r="C110" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>HIHO</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E111" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F111" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="G111" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G112" t="n">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F113" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G113" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>LMFA</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="E114" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="F114" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="G114" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>PKE</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>37.74</v>
+      </c>
+      <c r="E115" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="F115" t="n">
+        <v>44.29</v>
+      </c>
+      <c r="G115" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>RPT</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="E116" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="F116" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="G116" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="E117" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="F117" t="n">
+        <v>14.32</v>
+      </c>
+      <c r="G117" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="E118" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F118" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="G118" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>VIVS</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G119" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>AMC</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>FGMC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-23
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G206"/>
+  <dimension ref="A1:G225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5171,6 +5171,425 @@
         </is>
       </c>
       <c r="C206" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>CYCN</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="E207" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F207" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="G207" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>EVH</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="E208" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="F208" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="G208" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>GSHD</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>57.89</v>
+      </c>
+      <c r="E209" t="n">
+        <v>50.03</v>
+      </c>
+      <c r="F209" t="n">
+        <v>73.61</v>
+      </c>
+      <c r="G209" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>428.88</v>
+      </c>
+      <c r="E210" t="n">
+        <v>385.22</v>
+      </c>
+      <c r="F210" t="n">
+        <v>516.2</v>
+      </c>
+      <c r="G210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E211" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F211" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G211" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>RNAZ</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="E212" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F212" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="G212" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>20.75</v>
+      </c>
+      <c r="E213" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="F213" t="n">
+        <v>36.21</v>
+      </c>
+      <c r="G213" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E214" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="F214" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="G214" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>BWIN</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>FATE</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>HNGE</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>MSLE</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>RPD</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -5187,7 +5606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7996,6 +8415,374 @@
         </is>
       </c>
       <c r="C122" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="E123" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="F123" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="G123" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>AIRJ</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E124" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="F124" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="G124" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>ARWR</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>89.20999999999999</v>
+      </c>
+      <c r="E125" t="n">
+        <v>84.36</v>
+      </c>
+      <c r="F125" t="n">
+        <v>98.91</v>
+      </c>
+      <c r="G125" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>FNWD</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>43.88</v>
+      </c>
+      <c r="E126" t="n">
+        <v>43.12</v>
+      </c>
+      <c r="F126" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="G126" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>KUST</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="E127" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F127" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="G127" t="n">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>LABT</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="E128" t="n">
+        <v>3</v>
+      </c>
+      <c r="F128" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="G128" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>PAG</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>219.09</v>
+      </c>
+      <c r="E129" t="n">
+        <v>212.78</v>
+      </c>
+      <c r="F129" t="n">
+        <v>231.71</v>
+      </c>
+      <c r="G129" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>29.81</v>
+      </c>
+      <c r="E130" t="n">
+        <v>28.62</v>
+      </c>
+      <c r="F130" t="n">
+        <v>32.19</v>
+      </c>
+      <c r="G130" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>LMFA</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>PKE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>RPT</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>VIVS</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-24
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G225"/>
+  <dimension ref="A1:G240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5590,6 +5590,369 @@
         </is>
       </c>
       <c r="C225" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E226" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F226" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="G226" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>CIRC</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="E227" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G227" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>DAVE</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>458.25</v>
+      </c>
+      <c r="E228" t="n">
+        <v>383.48</v>
+      </c>
+      <c r="F228" t="n">
+        <v>607.79</v>
+      </c>
+      <c r="G228" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>FTH</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="E229" t="n">
+        <v>23.82</v>
+      </c>
+      <c r="F229" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="G229" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E230" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="F230" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="G230" t="n">
+        <v>1666</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>MNPR</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>116.64</v>
+      </c>
+      <c r="E231" t="n">
+        <v>97.93000000000001</v>
+      </c>
+      <c r="F231" t="n">
+        <v>154.05</v>
+      </c>
+      <c r="G231" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>PAY</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="E232" t="n">
+        <v>27.97</v>
+      </c>
+      <c r="F232" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="G232" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="E233" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="F233" t="n">
+        <v>18.39</v>
+      </c>
+      <c r="G233" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>10.48</v>
+      </c>
+      <c r="E234" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="F234" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="G234" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>EVH</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>GSHD</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>RNAZ</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -5606,7 +5969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8783,6 +9146,345 @@
         </is>
       </c>
       <c r="C138" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="E139" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="F139" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="G139" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>DOMO</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="E140" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="F140" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="G140" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="G141" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>MEDP</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>677.9</v>
+      </c>
+      <c r="E142" t="n">
+        <v>592.65</v>
+      </c>
+      <c r="F142" t="n">
+        <v>848.4</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>NEUP</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E143" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F143" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G143" t="n">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>NVEC</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>118.94</v>
+      </c>
+      <c r="E144" t="n">
+        <v>106.38</v>
+      </c>
+      <c r="F144" t="n">
+        <v>144.07</v>
+      </c>
+      <c r="G144" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>RELL</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>22.15</v>
+      </c>
+      <c r="E145" t="n">
+        <v>20.61</v>
+      </c>
+      <c r="F145" t="n">
+        <v>25.23</v>
+      </c>
+      <c r="G145" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>AIRJ</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>ARWR</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>FNWD</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>HIHO</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>KUST</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>LABT</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>PAG</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -8799,7 +9501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9023,6 +9725,35 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PRPL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="G10" t="n">
+        <v>172</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-25
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G240"/>
+  <dimension ref="A1:G259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5953,6 +5953,425 @@
         </is>
       </c>
       <c r="C240" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>BGMS</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E241" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F241" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G241" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CLYM</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>14.01</v>
+      </c>
+      <c r="E242" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="F242" t="n">
+        <v>18.01</v>
+      </c>
+      <c r="G242" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="E243" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F243" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="G243" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>FSLY</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>21.92</v>
+      </c>
+      <c r="E244" t="n">
+        <v>19.08</v>
+      </c>
+      <c r="F244" t="n">
+        <v>27.61</v>
+      </c>
+      <c r="G244" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>KFRC</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="E245" t="n">
+        <v>54.51</v>
+      </c>
+      <c r="F245" t="n">
+        <v>73.08</v>
+      </c>
+      <c r="G245" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="E246" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="F246" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="G246" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>OPRX</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="E247" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="F247" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="G247" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>279.49</v>
+      </c>
+      <c r="E248" t="n">
+        <v>259.48</v>
+      </c>
+      <c r="F248" t="n">
+        <v>319.51</v>
+      </c>
+      <c r="G248" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>CIRC</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>CYCN</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>FTH</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>MNPR</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -5969,7 +6388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9485,6 +9904,432 @@
         </is>
       </c>
       <c r="C153" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>3</v>
+      </c>
+      <c r="E154" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="F154" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="G154" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F155" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="G155" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>LSH</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G156" t="n">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E157" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G157" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E158" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F158" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="G158" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>NDLS</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="E159" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="F159" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="G159" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>SAFT</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="E160" t="n">
+        <v>102.87</v>
+      </c>
+      <c r="F160" t="n">
+        <v>104.01</v>
+      </c>
+      <c r="G160" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>THC</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>246.55</v>
+      </c>
+      <c r="E161" t="n">
+        <v>229.37</v>
+      </c>
+      <c r="F161" t="n">
+        <v>280.93</v>
+      </c>
+      <c r="G161" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="E162" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F162" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G162" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>WKC</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="E163" t="n">
+        <v>37.81</v>
+      </c>
+      <c r="F163" t="n">
+        <v>47.08</v>
+      </c>
+      <c r="G163" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>DOMO</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>MEDP</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>NEUP</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>NVEC</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>RELL</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-28
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G259"/>
+  <dimension ref="A1:G274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6372,6 +6372,333 @@
         </is>
       </c>
       <c r="C259" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>AMWL</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>13.45</v>
+      </c>
+      <c r="E260" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="F260" t="n">
+        <v>19.24</v>
+      </c>
+      <c r="G260" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>BWEN</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>5.52</v>
+      </c>
+      <c r="E261" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="F261" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="G261" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="E262" t="n">
+        <v>241.18</v>
+      </c>
+      <c r="F262" t="n">
+        <v>347.74</v>
+      </c>
+      <c r="G262" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>QDEL</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>19.03</v>
+      </c>
+      <c r="E263" t="n">
+        <v>15.55</v>
+      </c>
+      <c r="F263" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="G263" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>23.57</v>
+      </c>
+      <c r="E264" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="F264" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="G264" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>RFL</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="E265" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="F265" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="G265" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>ALIT</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>CLYM</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>KFRC</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>PAY</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>VRNS</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -6388,7 +6715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G171"/>
+  <dimension ref="A1:G187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10330,6 +10657,350 @@
         </is>
       </c>
       <c r="C171" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="E172" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="F172" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="G172" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="E173" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="F173" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G173" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>EDBL</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E174" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F174" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G174" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>FBRX</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>76.45999999999999</v>
+      </c>
+      <c r="E175" t="n">
+        <v>76.39</v>
+      </c>
+      <c r="F175" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="G175" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>GOSS</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E176" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G176" t="n">
+        <v>1773</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G177" t="n">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>LSH</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>NDLS</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>SAFT</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>THC</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>WKC</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-29
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G274"/>
+  <dimension ref="A1:G289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6699,6 +6699,333 @@
         </is>
       </c>
       <c r="C274" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>ANGX</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="E275" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="F275" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="G275" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>DCGO</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F276" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G276" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="E277" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F277" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="G277" t="n">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="E278" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="F278" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="G278" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>VRNS</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>49.54</v>
+      </c>
+      <c r="E279" t="n">
+        <v>44.29</v>
+      </c>
+      <c r="F279" t="n">
+        <v>60.04</v>
+      </c>
+      <c r="G279" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>VSTS</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="E280" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="F280" t="n">
+        <v>20.72</v>
+      </c>
+      <c r="G280" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>BGMS</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>BWEN</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>DAVE</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>FSLY</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>OPRX</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>QDEL</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>RFL</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -6715,7 +7042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G187"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11001,6 +11328,323 @@
         </is>
       </c>
       <c r="C187" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E188" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F188" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G188" t="n">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>14.12</v>
+      </c>
+      <c r="E189" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F189" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="G189" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>241.91</v>
+      </c>
+      <c r="E190" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="F190" t="n">
+        <v>260.72</v>
+      </c>
+      <c r="G190" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E191" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F191" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="G191" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E192" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G192" t="n">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>OPK</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="E193" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F193" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G193" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>POLA</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E194" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F194" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="G194" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>PRLD</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="E195" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F195" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="G195" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>EDBL</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>FBRX</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -11017,7 +11661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11270,6 +11914,81 @@
         <v>172</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DBGI</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="E11" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" t="n">
+        <v>36.69</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-13.38</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PRPL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-30
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G289"/>
+  <dimension ref="A1:G304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7026,6 +7026,369 @@
         </is>
       </c>
       <c r="C289" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>ATAI</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="E290" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="F290" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="G290" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>JTAI</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="E291" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F291" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="G291" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="E292" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F292" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="G292" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>MNPR</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>116.64</v>
+      </c>
+      <c r="E293" t="n">
+        <v>101</v>
+      </c>
+      <c r="F293" t="n">
+        <v>147.91</v>
+      </c>
+      <c r="G293" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>MRVI</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="E294" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="F294" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="G294" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>NXTC</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>7</v>
+      </c>
+      <c r="E295" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F295" t="n">
+        <v>12.98</v>
+      </c>
+      <c r="G295" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>SNAL</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="E296" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="F296" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="G296" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="E297" t="n">
+        <v>92.37</v>
+      </c>
+      <c r="F297" t="n">
+        <v>130.41</v>
+      </c>
+      <c r="G297" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>XWEL</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="E298" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F298" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="G298" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>ANGX</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>DCGO</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>VRNS</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>VSTS</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -7042,7 +7405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11645,6 +12008,507 @@
         </is>
       </c>
       <c r="C200" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="E201" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="F201" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="G201" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E202" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="F202" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="G202" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>CBZ</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>54.59</v>
+      </c>
+      <c r="E203" t="n">
+        <v>54.35</v>
+      </c>
+      <c r="F203" t="n">
+        <v>55.07</v>
+      </c>
+      <c r="G203" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>HURN</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>142.52</v>
+      </c>
+      <c r="E204" t="n">
+        <v>130.74</v>
+      </c>
+      <c r="F204" t="n">
+        <v>166.08</v>
+      </c>
+      <c r="G204" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>MANH</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>204.01</v>
+      </c>
+      <c r="E205" t="n">
+        <v>190.82</v>
+      </c>
+      <c r="F205" t="n">
+        <v>230.38</v>
+      </c>
+      <c r="G205" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>MWYN</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E206" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F206" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G206" t="n">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>NCRA</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="E207" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="F207" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="G207" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>NEO</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="E208" t="n">
+        <v>14.71</v>
+      </c>
+      <c r="F208" t="n">
+        <v>18.88</v>
+      </c>
+      <c r="G208" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>ONMD</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E209" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F209" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="G209" t="n">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>RCKY</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>50.41</v>
+      </c>
+      <c r="E210" t="n">
+        <v>47.42</v>
+      </c>
+      <c r="F210" t="n">
+        <v>56.39</v>
+      </c>
+      <c r="G210" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E211" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="F211" t="n">
+        <v>4</v>
+      </c>
+      <c r="G211" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>VRRM</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="E212" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="F212" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="G212" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>GOSS</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>IQV</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>OPK</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>POLA</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>PRLD</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -11661,7 +12525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11989,6 +12853,23 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DBGI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-07-31
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G304"/>
+  <dimension ref="A1:G311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7389,6 +7389,173 @@
         </is>
       </c>
       <c r="C304" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>57.08</v>
+      </c>
+      <c r="E305" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="F305" t="n">
+        <v>73.48</v>
+      </c>
+      <c r="G305" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>OSRH</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G306" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="E307" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="F307" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="G307" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="E308" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F308" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="G308" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>MNPR</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -7405,7 +7572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G221"/>
+  <dimension ref="A1:G245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12509,6 +12676,558 @@
         </is>
       </c>
       <c r="C221" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>BAX</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>30</v>
+      </c>
+      <c r="E222" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="F222" t="n">
+        <v>37.91</v>
+      </c>
+      <c r="G222" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>CMCO</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="E223" t="n">
+        <v>18.82</v>
+      </c>
+      <c r="F223" t="n">
+        <v>24.77</v>
+      </c>
+      <c r="G223" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>112.85</v>
+      </c>
+      <c r="E224" t="n">
+        <v>104.94</v>
+      </c>
+      <c r="F224" t="n">
+        <v>128.67</v>
+      </c>
+      <c r="G224" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E225" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F225" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G225" t="n">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E226" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F226" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G226" t="n">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>LUNG</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E227" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G227" t="n">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>MKTX</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>163.94</v>
+      </c>
+      <c r="E228" t="n">
+        <v>162.3</v>
+      </c>
+      <c r="F228" t="n">
+        <v>167.22</v>
+      </c>
+      <c r="G228" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>NUWE</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="E229" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F229" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="G229" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>SMHI</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="E230" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="F230" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="G230" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>SMTI</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="E231" t="n">
+        <v>33.35</v>
+      </c>
+      <c r="F231" t="n">
+        <v>34.81</v>
+      </c>
+      <c r="G231" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>VSEE</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E232" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F232" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G232" t="n">
+        <v>1953</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>XRX</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="E233" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F233" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="G233" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>CBZ</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>HURN</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>MANH</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>MWYN</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>NCRA</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>NEO</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>ONMD</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>RCKY</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>VRRM</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-01
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G311"/>
+  <dimension ref="A1:G324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7556,6 +7556,299 @@
         </is>
       </c>
       <c r="C311" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>MNPR</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>116.68</v>
+      </c>
+      <c r="E312" t="n">
+        <v>101</v>
+      </c>
+      <c r="F312" t="n">
+        <v>148.05</v>
+      </c>
+      <c r="G312" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>20.39</v>
+      </c>
+      <c r="E313" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="F313" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="G313" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>20</v>
+      </c>
+      <c r="E314" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="F314" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="G314" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="E315" t="n">
+        <v>92.37</v>
+      </c>
+      <c r="F315" t="n">
+        <v>130.41</v>
+      </c>
+      <c r="G315" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>VSTM</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="E316" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="F316" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G316" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>WRAP</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="E317" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F317" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="G317" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>INHD</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>JTAI</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>NXTC</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>XWEL</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -7572,7 +7865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G245"/>
+  <dimension ref="A1:G265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13228,6 +13521,442 @@
         </is>
       </c>
       <c r="C245" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>68.92</v>
+      </c>
+      <c r="E246" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="F246" t="n">
+        <v>95.54000000000001</v>
+      </c>
+      <c r="G246" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>FCUV</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="E247" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="F247" t="n">
+        <v>18.05</v>
+      </c>
+      <c r="G247" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>KUST</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="E248" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="F248" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="G248" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>MGRX</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E249" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F249" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="G249" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>NWL</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="E250" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F250" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G250" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E251" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G251" t="n">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>REPL</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="E252" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="F252" t="n">
+        <v>18.61</v>
+      </c>
+      <c r="G252" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>TCX</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="E253" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F253" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="G253" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>BAX</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>CMCO</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>LUNG</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>MKTX</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>NUWE</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>SMHI</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>SMTI</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>VSEE</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>XRX</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -13244,7 +13973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13589,6 +14318,23 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-04
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G324"/>
+  <dimension ref="A1:G337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7849,6 +7849,227 @@
         </is>
       </c>
       <c r="C324" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>AMWL</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>ATAI</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>CRNX</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>MNPR</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>MRVI</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>OSRH</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>SNAL</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>VSTM</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>WRAP</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -7865,7 +8086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13957,6 +14178,490 @@
         </is>
       </c>
       <c r="C265" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>ADGM</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E266" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F266" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G266" t="n">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>ATKR</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="E267" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="F267" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="G267" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>BOW</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>35.07</v>
+      </c>
+      <c r="E268" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="F268" t="n">
+        <v>38.21</v>
+      </c>
+      <c r="G268" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="E269" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F269" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="G269" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>EDBL</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E270" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F270" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G270" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>EZRA</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E271" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F271" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="G271" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>HYFM</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="E272" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F272" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="G272" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>RUBI</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="E273" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F273" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="G273" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>SDST</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E274" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F274" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G274" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="E275" t="n">
+        <v>44.17</v>
+      </c>
+      <c r="F275" t="n">
+        <v>69.16</v>
+      </c>
+      <c r="G275" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>XAIR</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E276" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="F276" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="G276" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>YYAI</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E277" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F277" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G277" t="n">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>FCUV</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>KUST</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>MGRX</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>NWL</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>REPL</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>TCX</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-05
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G337"/>
+  <dimension ref="A1:G343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8073,6 +8073,180 @@
         <is>
           <t>Dropped</t>
         </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>ATAI</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="E338" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="F338" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="G338" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>JSPR</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="E339" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F339" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G339" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="E340" t="n">
+        <v>14.39</v>
+      </c>
+      <c r="F340" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="G340" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>SUNE</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E341" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="F341" t="n">
+        <v>4</v>
+      </c>
+      <c r="G341" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>TXG</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>50.34</v>
+      </c>
+      <c r="E342" t="n">
+        <v>45.01</v>
+      </c>
+      <c r="F342" t="n">
+        <v>61</v>
+      </c>
+      <c r="G342" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="E343" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="F343" t="n">
+        <v>14.47</v>
+      </c>
+      <c r="G343" t="n">
+        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -8086,7 +8260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G285"/>
+  <dimension ref="A1:G316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14662,6 +14836,773 @@
         </is>
       </c>
       <c r="C285" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E286" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="F286" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="G286" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>AMRC</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>31.93</v>
+      </c>
+      <c r="E287" t="n">
+        <v>27.33</v>
+      </c>
+      <c r="F287" t="n">
+        <v>41.13</v>
+      </c>
+      <c r="G287" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>BLZE</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="E288" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="F288" t="n">
+        <v>32.67</v>
+      </c>
+      <c r="G288" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>BRCC</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="E289" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F289" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="G289" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>DDD</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="E290" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F290" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="G290" t="n">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>DORM</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>149.09</v>
+      </c>
+      <c r="E291" t="n">
+        <v>140</v>
+      </c>
+      <c r="F291" t="n">
+        <v>167.27</v>
+      </c>
+      <c r="G291" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>ENSC</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E292" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G292" t="n">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>IBTA</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>35.97</v>
+      </c>
+      <c r="E293" t="n">
+        <v>30.47</v>
+      </c>
+      <c r="F293" t="n">
+        <v>46.97</v>
+      </c>
+      <c r="G293" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>JELD</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="E294" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F294" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G294" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>LIFE</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>28.78</v>
+      </c>
+      <c r="E295" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="F295" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="G295" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>LSH</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E296" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G296" t="n">
+        <v>3012</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="E297" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="F297" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="G297" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>MOVE</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>18.07</v>
+      </c>
+      <c r="E298" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F298" t="n">
+        <v>27.19</v>
+      </c>
+      <c r="G298" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>NUWE</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="E299" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F299" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="G299" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>PAY</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>40.48</v>
+      </c>
+      <c r="E300" t="n">
+        <v>37.24</v>
+      </c>
+      <c r="F300" t="n">
+        <v>46.96</v>
+      </c>
+      <c r="G300" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>149.85</v>
+      </c>
+      <c r="E301" t="n">
+        <v>143.28</v>
+      </c>
+      <c r="F301" t="n">
+        <v>162.99</v>
+      </c>
+      <c r="G301" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>UFPT</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>331.54</v>
+      </c>
+      <c r="E302" t="n">
+        <v>305</v>
+      </c>
+      <c r="F302" t="n">
+        <v>384.62</v>
+      </c>
+      <c r="G302" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>VGAS</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E303" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F303" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G303" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>113.78</v>
+      </c>
+      <c r="E304" t="n">
+        <v>108</v>
+      </c>
+      <c r="F304" t="n">
+        <v>125.34</v>
+      </c>
+      <c r="G304" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>XGN</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="E305" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="F305" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="G305" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>ATKR</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>BOW</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>EDBL</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>EZRA</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>HYFM</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>RUBI</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>SDST</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>XAIR</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>YYAI</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-06
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G343"/>
+  <dimension ref="A1:G350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8247,6 +8247,185 @@
       </c>
       <c r="G343" t="n">
         <v>357</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>CIIT</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="E344" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F344" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="G344" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>CYCN</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="E345" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="F345" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="G345" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>JTAI</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="E346" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F346" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="G346" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>OSRH</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E347" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G347" t="n">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>16.98</v>
+      </c>
+      <c r="E348" t="n">
+        <v>15.85</v>
+      </c>
+      <c r="F348" t="n">
+        <v>19.24</v>
+      </c>
+      <c r="G348" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>SUNE</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8260,7 +8439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G316"/>
+  <dimension ref="A1:G349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15603,6 +15782,711 @@
         </is>
       </c>
       <c r="C316" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E317" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="F317" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="G317" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>BEEP</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="E318" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F318" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G318" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="E319" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F319" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G319" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>BLMN</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="E320" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="F320" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="G320" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E321" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G321" t="n">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>53.28</v>
+      </c>
+      <c r="E322" t="n">
+        <v>50.22</v>
+      </c>
+      <c r="F322" t="n">
+        <v>59.41</v>
+      </c>
+      <c r="G322" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>FTK</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>35.42</v>
+      </c>
+      <c r="E323" t="n">
+        <v>32.72</v>
+      </c>
+      <c r="F323" t="n">
+        <v>40.82</v>
+      </c>
+      <c r="G323" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>OESX</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="E324" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="F324" t="n">
+        <v>16.31</v>
+      </c>
+      <c r="G324" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>PRMB</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>25.87</v>
+      </c>
+      <c r="E325" t="n">
+        <v>24.43</v>
+      </c>
+      <c r="F325" t="n">
+        <v>28.75</v>
+      </c>
+      <c r="G325" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="E326" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="F326" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="G326" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>TBI</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="E327" t="n">
+        <v>9</v>
+      </c>
+      <c r="F327" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="G327" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>TVTX</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>63.84</v>
+      </c>
+      <c r="E328" t="n">
+        <v>61</v>
+      </c>
+      <c r="F328" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="G328" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>ADGM</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>AMRC</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>BLZE</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>BRCC</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>DDD</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>DORM</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>ENSC</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>IBTA</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>JELD</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>LIFE</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>LSH</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>MOVE</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>NUWE</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>PAY</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>UFPT</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>VGAS</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>XGN</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -15619,7 +16503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15981,6 +16865,35 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CSAI</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G16" t="n">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-07
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G350"/>
+  <dimension ref="A1:G358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8423,6 +8423,214 @@
         </is>
       </c>
       <c r="C350" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>FFAI</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="E351" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F351" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G351" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>LEDS</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="E352" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="F352" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="G352" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>19.91</v>
+      </c>
+      <c r="E353" t="n">
+        <v>15.46</v>
+      </c>
+      <c r="F353" t="n">
+        <v>28.81</v>
+      </c>
+      <c r="G353" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="E354" t="n">
+        <v>14.39</v>
+      </c>
+      <c r="F354" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="G354" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>20</v>
+      </c>
+      <c r="E355" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="F355" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="G355" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>SUNE</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E356" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="F356" t="n">
+        <v>4</v>
+      </c>
+      <c r="G356" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>CIIT</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>JSPR</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -8439,7 +8647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G349"/>
+  <dimension ref="A1:G385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16487,6 +16695,906 @@
         </is>
       </c>
       <c r="C349" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>AEVA</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>26.09</v>
+      </c>
+      <c r="E350" t="n">
+        <v>22.75</v>
+      </c>
+      <c r="F350" t="n">
+        <v>32.77</v>
+      </c>
+      <c r="G350" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>ASPN</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E351" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="F351" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="G351" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>ATNI</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>28.35</v>
+      </c>
+      <c r="E352" t="n">
+        <v>27.02</v>
+      </c>
+      <c r="F352" t="n">
+        <v>31.01</v>
+      </c>
+      <c r="G352" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>CAI</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="E353" t="n">
+        <v>17.94</v>
+      </c>
+      <c r="F353" t="n">
+        <v>22.61</v>
+      </c>
+      <c r="G353" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>CDRE</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>36</v>
+      </c>
+      <c r="E354" t="n">
+        <v>33.54</v>
+      </c>
+      <c r="F354" t="n">
+        <v>40.92</v>
+      </c>
+      <c r="G354" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>CELZ</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E355" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F355" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="G355" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="E356" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="F356" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="G356" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>DCTH</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>15.44</v>
+      </c>
+      <c r="E357" t="n">
+        <v>14.03</v>
+      </c>
+      <c r="F357" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="G357" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>ENSC</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E358" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F358" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G358" t="n">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>EOLS</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>7</v>
+      </c>
+      <c r="E359" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="F359" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="G359" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>HNST</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="E360" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="F360" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="G360" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="E361" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F361" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="G361" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>INSM</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>132.25</v>
+      </c>
+      <c r="E362" t="n">
+        <v>126.48</v>
+      </c>
+      <c r="F362" t="n">
+        <v>143.79</v>
+      </c>
+      <c r="G362" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="E363" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="F363" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="G363" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>KRO</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="E364" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F364" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="G364" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>MGNI</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>25.13</v>
+      </c>
+      <c r="E365" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="F365" t="n">
+        <v>30.19</v>
+      </c>
+      <c r="G365" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>MGRX</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E366" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G366" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="E367" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F367" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="G367" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>OPRT</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E368" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="F368" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="G368" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>PAYC</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>216</v>
+      </c>
+      <c r="E369" t="n">
+        <v>208</v>
+      </c>
+      <c r="F369" t="n">
+        <v>232</v>
+      </c>
+      <c r="G369" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>SNOA</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E370" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F370" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="G370" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E371" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F371" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G371" t="n">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>TASK</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="E372" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="F372" t="n">
+        <v>8.07</v>
+      </c>
+      <c r="G372" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>TRUP</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>29.08</v>
+      </c>
+      <c r="E373" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F373" t="n">
+        <v>34.65</v>
+      </c>
+      <c r="G373" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>BEEP</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>BLMN</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>FTK</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>OESX</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>PRMB</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>TBI</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>TVTX</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-10
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G370"/>
+  <dimension ref="A1:G374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8895,6 +8895,74 @@
         </is>
       </c>
       <c r="C370" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>LPRO</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>OSRH</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -8911,7 +8979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G430"/>
+  <dimension ref="A1:G470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18900,6 +18968,866 @@
         </is>
       </c>
       <c r="C430" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>ACHR</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E431" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="F431" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="G431" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="E432" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="F432" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="G432" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>AQST</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="E433" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="F433" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="G433" t="n">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>AUUD</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="E434" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F434" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="G434" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>42.44</v>
+      </c>
+      <c r="E435" t="n">
+        <v>42.17</v>
+      </c>
+      <c r="F435" t="n">
+        <v>42.98</v>
+      </c>
+      <c r="G435" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>CHMI</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="E436" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F436" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="G436" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>FEAM</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="E437" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F437" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="G437" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>HZO</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>51.95</v>
+      </c>
+      <c r="E438" t="n">
+        <v>51.87</v>
+      </c>
+      <c r="F438" t="n">
+        <v>52.11</v>
+      </c>
+      <c r="G438" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>POWW</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E439" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="F439" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="G439" t="n">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E440" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F440" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G440" t="n">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>SCKT</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="E441" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F441" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="G441" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>TOI</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="E442" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="F442" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="G442" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E443" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F443" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="G443" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="E444" t="n">
+        <v>18.36</v>
+      </c>
+      <c r="F444" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G444" t="n">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="E445" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="F445" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="G445" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>AQB</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>CART</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>CELZ</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>CRSR</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>DOCS</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>EMBC</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>FIGS</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>FNKO</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>FOXF</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>GTN</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>INOD</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>MTW</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>NRXP</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>PUBM</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>QNST</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>SENS</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>THRY</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>TWLO</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>UEIC</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>VATE</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>ZENA</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -18916,7 +19844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19307,6 +20235,23 @@
         <v>33</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CSAI</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-11
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G374"/>
+  <dimension ref="A1:G381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8963,6 +8963,185 @@
         </is>
       </c>
       <c r="C374" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>AGEN</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="E375" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="F375" t="n">
+        <v>13.83</v>
+      </c>
+      <c r="G375" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>59.67</v>
+      </c>
+      <c r="E376" t="n">
+        <v>54.09</v>
+      </c>
+      <c r="F376" t="n">
+        <v>70.83</v>
+      </c>
+      <c r="G376" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>CDT</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="E377" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F377" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="G377" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>PRPL</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>10</v>
+      </c>
+      <c r="E378" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="F378" t="n">
+        <v>17.54</v>
+      </c>
+      <c r="G378" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="E379" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="F379" t="n">
+        <v>27.01</v>
+      </c>
+      <c r="G379" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>JTAI</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -8979,7 +9158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G470"/>
+  <dimension ref="A1:G496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19828,6 +20007,580 @@
         </is>
       </c>
       <c r="C470" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="E471" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="F471" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="G471" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>AIHS</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="E472" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F472" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="G472" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="E473" t="n">
+        <v>9</v>
+      </c>
+      <c r="F473" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="G473" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>FENC</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="E474" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="F474" t="n">
+        <v>16.53</v>
+      </c>
+      <c r="G474" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>GENK</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E475" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="F475" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="G475" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>NCRA</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D476" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="E476" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="F476" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="G476" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>PLBY</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E477" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F477" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="G477" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>16.64</v>
+      </c>
+      <c r="E478" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="F478" t="n">
+        <v>21.94</v>
+      </c>
+      <c r="G478" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>RIOT</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>23.66</v>
+      </c>
+      <c r="E479" t="n">
+        <v>19.34</v>
+      </c>
+      <c r="F479" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="G479" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>STIM</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="E480" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F480" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="G480" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>TISI</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>21</v>
+      </c>
+      <c r="E481" t="n">
+        <v>18.68</v>
+      </c>
+      <c r="F481" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="G481" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>ACHR</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>AQST</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>AUUD</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>CHMI</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>FEAM</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>HZO</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>POWW</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>SCKT</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>TOI</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-12
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G381"/>
+  <dimension ref="A1:G387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9142,6 +9142,156 @@
         </is>
       </c>
       <c r="C381" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="E382" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="F382" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="G382" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="E383" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="F383" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G383" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>JTAI</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E384" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F384" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="G384" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>19.98</v>
+      </c>
+      <c r="E385" t="n">
+        <v>15.46</v>
+      </c>
+      <c r="F385" t="n">
+        <v>29.02</v>
+      </c>
+      <c r="G385" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>AGEN</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -9158,7 +9308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G496"/>
+  <dimension ref="A1:G518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20581,6 +20731,512 @@
         </is>
       </c>
       <c r="C496" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>AII</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>25</v>
+      </c>
+      <c r="E497" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="F497" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="G497" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="E498" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F498" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="G498" t="n">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>BOXL</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="E499" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="F499" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="G499" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>CAVA</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>71</v>
+      </c>
+      <c r="E500" t="n">
+        <v>67.03</v>
+      </c>
+      <c r="F500" t="n">
+        <v>78.94</v>
+      </c>
+      <c r="G500" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>DOGZ</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E501" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F501" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="G501" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>DRMA</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="E502" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F502" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G502" t="n">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>FEMY</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E503" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F503" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G503" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>GRWG</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E504" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F504" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G504" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>HRB</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="E505" t="n">
+        <v>52.29</v>
+      </c>
+      <c r="F505" t="n">
+        <v>61.62</v>
+      </c>
+      <c r="G505" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>RMCF</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E506" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F506" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="G506" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="E507" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="F507" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="G507" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>AIHS</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>FENC</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>GENK</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>NCRA</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>PLBY</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>RIOT</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>STIM</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>TISI</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-13
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G387"/>
+  <dimension ref="A1:G400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9292,6 +9292,311 @@
         </is>
       </c>
       <c r="C387" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="E388" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="F388" t="n">
+        <v>17.29</v>
+      </c>
+      <c r="G388" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="E389" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F389" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="G389" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>118.53</v>
+      </c>
+      <c r="E390" t="n">
+        <v>107.32</v>
+      </c>
+      <c r="F390" t="n">
+        <v>140.95</v>
+      </c>
+      <c r="G390" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>DBGI</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>30.93</v>
+      </c>
+      <c r="E391" t="n">
+        <v>11.83</v>
+      </c>
+      <c r="F391" t="n">
+        <v>69.13</v>
+      </c>
+      <c r="G391" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>70.78</v>
+      </c>
+      <c r="E392" t="n">
+        <v>22.72</v>
+      </c>
+      <c r="F392" t="n">
+        <v>166.9</v>
+      </c>
+      <c r="G392" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>72.64</v>
+      </c>
+      <c r="E393" t="n">
+        <v>62.68</v>
+      </c>
+      <c r="F393" t="n">
+        <v>92.56</v>
+      </c>
+      <c r="G393" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>NDLS</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>19</v>
+      </c>
+      <c r="E394" t="n">
+        <v>15.58</v>
+      </c>
+      <c r="F394" t="n">
+        <v>25.84</v>
+      </c>
+      <c r="G394" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>CDT</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>JTAI</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>PRPL</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -9308,7 +9613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G518"/>
+  <dimension ref="A1:G543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21237,6 +21542,599 @@
         </is>
       </c>
       <c r="C518" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>AIRO</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="E519" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F519" t="n">
+        <v>15.54</v>
+      </c>
+      <c r="G519" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>10.11</v>
+      </c>
+      <c r="E520" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="F520" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="G520" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>CHCI</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>18</v>
+      </c>
+      <c r="E521" t="n">
+        <v>16.13</v>
+      </c>
+      <c r="F521" t="n">
+        <v>21.74</v>
+      </c>
+      <c r="G521" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>CRMD</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="E522" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="F522" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="G522" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>CURI</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D523" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="E523" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="F523" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="G523" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>DFSC</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D524" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="E524" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="F524" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G524" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>GXAI</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D525" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="E525" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F525" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="G525" t="n">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>HLIT</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D526" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="E526" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="F526" t="n">
+        <v>19.66</v>
+      </c>
+      <c r="G526" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>IVDA</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D527" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E527" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G527" t="n">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>LIMN</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E528" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F528" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G528" t="n">
+        <v>2202</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>LNSR</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="E529" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="F529" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="G529" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>17.94</v>
+      </c>
+      <c r="E530" t="n">
+        <v>16.27</v>
+      </c>
+      <c r="F530" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="G530" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>PAVM</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E531" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="F531" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="G531" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>USIO</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="E532" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F532" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G532" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>AII</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>BOXL</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>CAVA</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>DOGZ</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>DRMA</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>FEMY</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>GRWG</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>HRB</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>RMCF</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-14
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G400"/>
+  <dimension ref="A1:G409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9597,6 +9597,219 @@
         </is>
       </c>
       <c r="C400" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>CDT</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="E401" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F401" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="G401" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="E402" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="F402" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G402" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="E403" t="n">
+        <v>14.54</v>
+      </c>
+      <c r="F403" t="n">
+        <v>29.12</v>
+      </c>
+      <c r="G403" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>PRPL</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>10</v>
+      </c>
+      <c r="E404" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="F404" t="n">
+        <v>17.54</v>
+      </c>
+      <c r="G404" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>SMTI</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>34.39</v>
+      </c>
+      <c r="E405" t="n">
+        <v>33.68</v>
+      </c>
+      <c r="F405" t="n">
+        <v>35.81</v>
+      </c>
+      <c r="G405" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>NDLS</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -9613,7 +9826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G543"/>
+  <dimension ref="A1:G571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22135,6 +22348,662 @@
         </is>
       </c>
       <c r="C543" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>BRUN</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D544" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="E544" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="F544" t="n">
+        <v>36.84</v>
+      </c>
+      <c r="G544" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="E545" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="F545" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="G545" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="E546" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="F546" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="G546" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>DARE</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="E547" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F547" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G547" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>59.69</v>
+      </c>
+      <c r="E548" t="n">
+        <v>53.01</v>
+      </c>
+      <c r="F548" t="n">
+        <v>73.06</v>
+      </c>
+      <c r="G548" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E549" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="F549" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="G549" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>39.88</v>
+      </c>
+      <c r="E550" t="n">
+        <v>36.04</v>
+      </c>
+      <c r="F550" t="n">
+        <v>47.57</v>
+      </c>
+      <c r="G550" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>IMXI</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="E551" t="n">
+        <v>13.71</v>
+      </c>
+      <c r="F551" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="G551" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>NXGL</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E552" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G552" t="n">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="E553" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F553" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="G553" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>34.29</v>
+      </c>
+      <c r="E554" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="F554" t="n">
+        <v>38.39</v>
+      </c>
+      <c r="G554" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>180.95</v>
+      </c>
+      <c r="E555" t="n">
+        <v>174</v>
+      </c>
+      <c r="F555" t="n">
+        <v>194.85</v>
+      </c>
+      <c r="G555" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>SKYE</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E556" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="F556" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G556" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D557" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E557" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F557" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G557" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>TPCS</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="E558" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="F558" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="G558" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>AIRO</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>CHCI</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>CRMD</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>CURI</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>GXAI</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>HLIT</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>IVDA</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>LIMN</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>LNSR</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>PAVM</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>USIO</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-17
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G409"/>
+  <dimension ref="A1:G422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9810,6 +9810,299 @@
         </is>
       </c>
       <c r="C409" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>49.76</v>
+      </c>
+      <c r="E410" t="n">
+        <v>44.54</v>
+      </c>
+      <c r="F410" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="G410" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E411" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F411" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G411" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>FATN</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="E412" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="F412" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="G412" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>FCUV</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>14.32</v>
+      </c>
+      <c r="E413" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="F413" t="n">
+        <v>33.22</v>
+      </c>
+      <c r="G413" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>11</v>
+      </c>
+      <c r="E414" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="F414" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="G414" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E415" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="F415" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="G415" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>DFNS</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>FFAI</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>LVLU</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>PRPL</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -9826,7 +10119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G571"/>
+  <dimension ref="A1:G597"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23004,6 +23297,580 @@
         </is>
       </c>
       <c r="C571" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>CNXU</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="E572" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="F572" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="G572" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>DUOT</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="E573" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F573" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="G573" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>FIEE</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="E574" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="F574" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="G574" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>IPST</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="E575" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="F575" t="n">
+        <v>13.82</v>
+      </c>
+      <c r="G575" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>IVF</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="E576" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="F576" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G576" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>MYSZ</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E577" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="F577" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="G577" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="E578" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F578" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="G578" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>PFSA</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="E579" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F579" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="G579" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>SLE</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="E580" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F580" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="G580" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="E581" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F581" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="G581" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="E582" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F582" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="G582" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>BRUN</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>DARE</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>DFSC</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>IMXI</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>NXGL</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>ONFO</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>TPCS</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-18
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G422"/>
+  <dimension ref="A1:G442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10103,6 +10103,526 @@
         </is>
       </c>
       <c r="C422" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>AAOI</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>160.99</v>
+      </c>
+      <c r="E423" t="n">
+        <v>118.88</v>
+      </c>
+      <c r="F423" t="n">
+        <v>245.21</v>
+      </c>
+      <c r="G423" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E424" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="F424" t="n">
+        <v>16.35</v>
+      </c>
+      <c r="G424" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E425" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F425" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="G425" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>AGL</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>114.32</v>
+      </c>
+      <c r="E426" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="F426" t="n">
+        <v>171.16</v>
+      </c>
+      <c r="G426" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>ANTX</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>7.19</v>
+      </c>
+      <c r="E427" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="F427" t="n">
+        <v>10.41</v>
+      </c>
+      <c r="G427" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>15.34</v>
+      </c>
+      <c r="E428" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="F428" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G428" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>ASBP</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="E429" t="n">
+        <v>6.89</v>
+      </c>
+      <c r="F429" t="n">
+        <v>10.36</v>
+      </c>
+      <c r="G429" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>BLZE</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>20.91</v>
+      </c>
+      <c r="E430" t="n">
+        <v>17.47</v>
+      </c>
+      <c r="F430" t="n">
+        <v>27.79</v>
+      </c>
+      <c r="G430" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="E431" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F431" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="G431" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>EFOR</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>33.78</v>
+      </c>
+      <c r="E432" t="n">
+        <v>30.18</v>
+      </c>
+      <c r="F432" t="n">
+        <v>40.98</v>
+      </c>
+      <c r="G432" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="E433" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="F433" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="G433" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>JELD</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="E434" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F434" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="G434" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>240.18</v>
+      </c>
+      <c r="E435" t="n">
+        <v>201.74</v>
+      </c>
+      <c r="F435" t="n">
+        <v>317.06</v>
+      </c>
+      <c r="G435" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>NDLS</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>18.65</v>
+      </c>
+      <c r="E436" t="n">
+        <v>15.52</v>
+      </c>
+      <c r="F436" t="n">
+        <v>24.91</v>
+      </c>
+      <c r="G436" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>18.85</v>
+      </c>
+      <c r="E437" t="n">
+        <v>15.32</v>
+      </c>
+      <c r="F437" t="n">
+        <v>25.91</v>
+      </c>
+      <c r="G437" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>DBGI</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>FCUV</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>SMTI</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -10119,7 +10639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G597"/>
+  <dimension ref="A1:G614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23871,6 +24391,403 @@
         </is>
       </c>
       <c r="C597" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>AEI</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E598" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F598" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="G598" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>AIXC</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="E599" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F599" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="G599" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>30.69</v>
+      </c>
+      <c r="E600" t="n">
+        <v>28</v>
+      </c>
+      <c r="F600" t="n">
+        <v>36.07</v>
+      </c>
+      <c r="G600" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E601" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F601" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G601" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>FLXS</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>84</v>
+      </c>
+      <c r="E602" t="n">
+        <v>76.18000000000001</v>
+      </c>
+      <c r="F602" t="n">
+        <v>99.64</v>
+      </c>
+      <c r="G602" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>SGLY</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="E603" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F603" t="n">
+        <v>13.69</v>
+      </c>
+      <c r="G603" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>SIEB</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="E604" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F604" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="G604" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>WEAV</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="E605" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="F605" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="G605" t="n">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>XOS</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E606" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F606" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="G606" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>CNXU</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>FIEE</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>IPST</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>IVF</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>MYSZ</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>SKYE</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -23887,7 +24804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24295,6 +25212,35 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IPST</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="E18" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-30.67</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-19
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G442"/>
+  <dimension ref="A1:G459"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10623,6 +10623,355 @@
         </is>
       </c>
       <c r="C442" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>97.79000000000001</v>
+      </c>
+      <c r="E443" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="F443" t="n">
+        <v>158.97</v>
+      </c>
+      <c r="G443" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="E444" t="n">
+        <v>14.93</v>
+      </c>
+      <c r="F444" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="G444" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>QXL</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="E445" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="F445" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="G445" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E446" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="F446" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="G446" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>TVGN</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>7</v>
+      </c>
+      <c r="E447" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F447" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G447" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>AAOI</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>ADVB</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>AGL</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>ASBP</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>BLZE</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>CDT</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>JELD</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>NDLS</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -10639,7 +10988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G614"/>
+  <dimension ref="A1:G640"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24788,6 +25137,604 @@
         </is>
       </c>
       <c r="C614" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>ARCT</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D615" t="n">
+        <v>10.97</v>
+      </c>
+      <c r="E615" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="F615" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="G615" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D616" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="E616" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F616" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="G616" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>EL</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D617" t="n">
+        <v>97.91</v>
+      </c>
+      <c r="E617" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="F617" t="n">
+        <v>106.74</v>
+      </c>
+      <c r="G617" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>FEMY</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="E618" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="F618" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="G618" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>122.25</v>
+      </c>
+      <c r="E619" t="n">
+        <v>114.46</v>
+      </c>
+      <c r="F619" t="n">
+        <v>137.83</v>
+      </c>
+      <c r="G619" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>MRVI</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="E620" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="F620" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="G620" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E621" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="F621" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G621" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>OPENZ</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E622" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F622" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G622" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>59.04</v>
+      </c>
+      <c r="E623" t="n">
+        <v>54.81</v>
+      </c>
+      <c r="F623" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="G623" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>TGL</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="E624" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F624" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G624" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>TNON</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="E625" t="n">
+        <v>9.890000000000001</v>
+      </c>
+      <c r="F625" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="G625" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>VRCA</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="E626" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="F626" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="G626" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="E627" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="F627" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="G627" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>AEI</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>AIXC</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>DUOT</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>FLXS</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>PFSA</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>SGLY</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>SIEB</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>SLE</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>WEAV</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>XOS</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -24804,7 +25751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25241,6 +26188,23 @@
         <v>2</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IPST</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-20
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G459"/>
+  <dimension ref="A1:G478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10972,6 +10972,473 @@
         </is>
       </c>
       <c r="C459" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>AAOI</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D460" t="n">
+        <v>160.99</v>
+      </c>
+      <c r="E460" t="n">
+        <v>118.6</v>
+      </c>
+      <c r="F460" t="n">
+        <v>245.77</v>
+      </c>
+      <c r="G460" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>ARTV</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D461" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="E461" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F461" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="G461" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>CSAI</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="E462" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="F462" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="G462" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="E463" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="F463" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="G463" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>FWRD</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D464" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="E464" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="F464" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="G464" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="E465" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F465" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="G465" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>NAVN</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D466" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="E466" t="n">
+        <v>28.16</v>
+      </c>
+      <c r="F466" t="n">
+        <v>33.65</v>
+      </c>
+      <c r="G466" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>196.72</v>
+      </c>
+      <c r="E467" t="n">
+        <v>178.26</v>
+      </c>
+      <c r="F467" t="n">
+        <v>233.64</v>
+      </c>
+      <c r="G467" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>SEGG</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="E468" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F468" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="G468" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>341.95</v>
+      </c>
+      <c r="E469" t="n">
+        <v>316.32</v>
+      </c>
+      <c r="F469" t="n">
+        <v>393.21</v>
+      </c>
+      <c r="G469" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E470" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="F470" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="G470" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="E471" t="n">
+        <v>14.11</v>
+      </c>
+      <c r="F471" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="G471" t="n">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>QTTB</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>QXL</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>TVGN</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -10988,7 +11455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G640"/>
+  <dimension ref="A1:G656"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25735,6 +26202,326 @@
         </is>
       </c>
       <c r="C640" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>BEEM</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E641" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F641" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="G641" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="E642" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F642" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G642" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>SCSC</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>66.78</v>
+      </c>
+      <c r="E643" t="n">
+        <v>56</v>
+      </c>
+      <c r="F643" t="n">
+        <v>88.34</v>
+      </c>
+      <c r="G643" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>SGLY</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E644" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F644" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="G644" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>ARCT</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>EL</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>FEMY</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>MRVI</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>OPENZ</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>TGL</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>TNON</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>VRCA</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-21
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G478"/>
+  <dimension ref="A1:G493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11439,6 +11439,321 @@
         </is>
       </c>
       <c r="C478" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>42.64</v>
+      </c>
+      <c r="E479" t="n">
+        <v>42.15</v>
+      </c>
+      <c r="F479" t="n">
+        <v>43.62</v>
+      </c>
+      <c r="G479" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>48.77</v>
+      </c>
+      <c r="E480" t="n">
+        <v>41.22</v>
+      </c>
+      <c r="F480" t="n">
+        <v>63.87</v>
+      </c>
+      <c r="G480" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>HZO</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>52.46</v>
+      </c>
+      <c r="E481" t="n">
+        <v>51.87</v>
+      </c>
+      <c r="F481" t="n">
+        <v>53.64</v>
+      </c>
+      <c r="G481" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D482" t="n">
+        <v>69.94</v>
+      </c>
+      <c r="E482" t="n">
+        <v>65.01000000000001</v>
+      </c>
+      <c r="F482" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="G482" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>18.63</v>
+      </c>
+      <c r="E483" t="n">
+        <v>18.36</v>
+      </c>
+      <c r="F483" t="n">
+        <v>19.16</v>
+      </c>
+      <c r="G483" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>AAOI</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>ARTV</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>EFOR</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>SEGG</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -11455,7 +11770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G656"/>
+  <dimension ref="A1:G663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26522,6 +26837,161 @@
         </is>
       </c>
       <c r="C656" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="E657" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F657" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="G657" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E658" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F658" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G658" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="E659" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F659" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="G659" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>BEEM</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>LOOP</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>SCSC</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>SGLY</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>